<commit_message>
Fix bulk-import: blank Link Object ID and Story ID to avoid format errors
https://claude.ai/code/session_01PamzbAcKurpbQ29kpfFhzA
</commit_message>
<xml_diff>
--- a/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
+++ b/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
@@ -989,7 +989,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>META_Leads_Recompo_Agenda_2026Q2</t>
@@ -1000,8 +999,6 @@
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Outcome Leads</t>
@@ -1012,19 +1009,11 @@
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1035,35 +1024,21 @@
           <t>Prospeccion_Broad_GrupoA</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>&lt;TU_PAGE_ID&gt;</t>
-        </is>
-      </c>
       <c r="X2" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
           <t>ES, CL, UY, CR, PR, US</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
           <t>All</t>
@@ -1079,31 +1054,11 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr">
         <is>
           <t>Spanish</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
       <c r="BD2" t="inlineStr">
         <is>
           <t>OFFSITE_CONVERSIONS</t>
@@ -1114,42 +1069,11 @@
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr"/>
-      <c r="BW2" t="inlineStr"/>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr"/>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr"/>
-      <c r="CC2" t="inlineStr"/>
-      <c r="CD2" t="inlineStr"/>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="inlineStr"/>
-      <c r="CH2" t="inlineStr"/>
-      <c r="CI2" t="inlineStr"/>
-      <c r="CJ2" t="inlineStr"/>
-      <c r="CK2" t="inlineStr"/>
       <c r="CL2" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1183,7 +1107,6 @@
           <t>salchichapro.com</t>
         </is>
       </c>
-      <c r="CR2" t="inlineStr"/>
       <c r="CS2" t="inlineStr">
         <is>
           <t>Video Page Post Ad</t>
@@ -1194,29 +1117,13 @@
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=recompo_agenda&amp;utm_content={{ad.name}}&amp;utm_term={{adset.name}}</t>
         </is>
       </c>
-      <c r="CU2" t="inlineStr"/>
-      <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr"/>
-      <c r="CX2" t="inlineStr"/>
-      <c r="CY2" t="inlineStr"/>
-      <c r="CZ2" t="inlineStr"/>
-      <c r="DA2" t="inlineStr"/>
-      <c r="DB2" t="inlineStr"/>
-      <c r="DC2" t="inlineStr"/>
-      <c r="DD2" t="inlineStr"/>
-      <c r="DE2" t="inlineStr"/>
-      <c r="DF2" t="inlineStr"/>
-      <c r="DG2" t="inlineStr"/>
-      <c r="DH2" t="inlineStr"/>
       <c r="DI2" t="inlineStr">
         <is>
           <t>LEARN_MORE</t>
         </is>
       </c>
-      <c r="DJ2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>META_Leads_Recompo_Agenda_2026Q2</t>
@@ -1227,8 +1134,6 @@
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>Outcome Leads</t>
@@ -1239,19 +1144,11 @@
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1262,35 +1159,21 @@
           <t>Prospeccion_Broad_GrupoA</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>&lt;TU_PAGE_ID&gt;</t>
-        </is>
-      </c>
       <c r="X3" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr">
         <is>
           <t>ES, CL, UY, CR, PR, US</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
           <t>All</t>
@@ -1306,31 +1189,11 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr">
         <is>
           <t>Spanish</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
       <c r="BD3" t="inlineStr">
         <is>
           <t>OFFSITE_CONVERSIONS</t>
@@ -1341,42 +1204,11 @@
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="BH3" t="inlineStr"/>
-      <c r="BI3" t="inlineStr"/>
-      <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="inlineStr"/>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr"/>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
-      <c r="BQ3" t="inlineStr"/>
-      <c r="BR3" t="inlineStr"/>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="inlineStr"/>
-      <c r="BU3" t="inlineStr"/>
-      <c r="BV3" t="inlineStr"/>
-      <c r="BW3" t="inlineStr"/>
-      <c r="BX3" t="inlineStr"/>
-      <c r="BY3" t="inlineStr"/>
-      <c r="BZ3" t="inlineStr"/>
-      <c r="CA3" t="inlineStr"/>
-      <c r="CB3" t="inlineStr"/>
-      <c r="CC3" t="inlineStr"/>
-      <c r="CD3" t="inlineStr"/>
-      <c r="CE3" t="inlineStr"/>
-      <c r="CF3" t="inlineStr"/>
-      <c r="CG3" t="inlineStr"/>
-      <c r="CH3" t="inlineStr"/>
-      <c r="CI3" t="inlineStr"/>
-      <c r="CJ3" t="inlineStr"/>
-      <c r="CK3" t="inlineStr"/>
       <c r="CL3" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1410,7 +1242,6 @@
           <t>salchichapro.com</t>
         </is>
       </c>
-      <c r="CR3" t="inlineStr"/>
       <c r="CS3" t="inlineStr">
         <is>
           <t>Video Page Post Ad</t>
@@ -1421,29 +1252,13 @@
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=recompo_agenda&amp;utm_content={{ad.name}}&amp;utm_term={{adset.name}}</t>
         </is>
       </c>
-      <c r="CU3" t="inlineStr"/>
-      <c r="CV3" t="inlineStr"/>
-      <c r="CW3" t="inlineStr"/>
-      <c r="CX3" t="inlineStr"/>
-      <c r="CY3" t="inlineStr"/>
-      <c r="CZ3" t="inlineStr"/>
-      <c r="DA3" t="inlineStr"/>
-      <c r="DB3" t="inlineStr"/>
-      <c r="DC3" t="inlineStr"/>
-      <c r="DD3" t="inlineStr"/>
-      <c r="DE3" t="inlineStr"/>
-      <c r="DF3" t="inlineStr"/>
-      <c r="DG3" t="inlineStr"/>
-      <c r="DH3" t="inlineStr"/>
       <c r="DI3" t="inlineStr">
         <is>
           <t>LEARN_MORE</t>
         </is>
       </c>
-      <c r="DJ3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>META_Leads_Recompo_Agenda_2026Q2</t>
@@ -1454,8 +1269,6 @@
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Outcome Leads</t>
@@ -1466,19 +1279,11 @@
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1489,35 +1294,21 @@
           <t>Prospeccion_Broad_GrupoA</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>&lt;TU_PAGE_ID&gt;</t>
-        </is>
-      </c>
       <c r="X4" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr">
         <is>
           <t>ES, CL, UY, CR, PR, US</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
           <t>All</t>
@@ -1533,31 +1324,11 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
       <c r="AQ4" t="inlineStr">
         <is>
           <t>Spanish</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
-      <c r="BB4" t="inlineStr"/>
-      <c r="BC4" t="inlineStr"/>
       <c r="BD4" t="inlineStr">
         <is>
           <t>OFFSITE_CONVERSIONS</t>
@@ -1568,42 +1339,11 @@
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="BH4" t="inlineStr"/>
-      <c r="BI4" t="inlineStr"/>
-      <c r="BJ4" t="inlineStr"/>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="inlineStr"/>
-      <c r="BM4" t="inlineStr"/>
-      <c r="BN4" t="inlineStr"/>
-      <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr"/>
-      <c r="BQ4" t="inlineStr"/>
-      <c r="BR4" t="inlineStr"/>
-      <c r="BS4" t="inlineStr"/>
-      <c r="BT4" t="inlineStr"/>
-      <c r="BU4" t="inlineStr"/>
-      <c r="BV4" t="inlineStr"/>
-      <c r="BW4" t="inlineStr"/>
-      <c r="BX4" t="inlineStr"/>
-      <c r="BY4" t="inlineStr"/>
-      <c r="BZ4" t="inlineStr"/>
-      <c r="CA4" t="inlineStr"/>
-      <c r="CB4" t="inlineStr"/>
-      <c r="CC4" t="inlineStr"/>
-      <c r="CD4" t="inlineStr"/>
-      <c r="CE4" t="inlineStr"/>
-      <c r="CF4" t="inlineStr"/>
-      <c r="CG4" t="inlineStr"/>
-      <c r="CH4" t="inlineStr"/>
-      <c r="CI4" t="inlineStr"/>
-      <c r="CJ4" t="inlineStr"/>
-      <c r="CK4" t="inlineStr"/>
       <c r="CL4" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1637,7 +1377,6 @@
           <t>salchichapro.com</t>
         </is>
       </c>
-      <c r="CR4" t="inlineStr"/>
       <c r="CS4" t="inlineStr">
         <is>
           <t>Video Page Post Ad</t>
@@ -1648,29 +1387,13 @@
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=recompo_agenda&amp;utm_content={{ad.name}}&amp;utm_term={{adset.name}}</t>
         </is>
       </c>
-      <c r="CU4" t="inlineStr"/>
-      <c r="CV4" t="inlineStr"/>
-      <c r="CW4" t="inlineStr"/>
-      <c r="CX4" t="inlineStr"/>
-      <c r="CY4" t="inlineStr"/>
-      <c r="CZ4" t="inlineStr"/>
-      <c r="DA4" t="inlineStr"/>
-      <c r="DB4" t="inlineStr"/>
-      <c r="DC4" t="inlineStr"/>
-      <c r="DD4" t="inlineStr"/>
-      <c r="DE4" t="inlineStr"/>
-      <c r="DF4" t="inlineStr"/>
-      <c r="DG4" t="inlineStr"/>
-      <c r="DH4" t="inlineStr"/>
       <c r="DI4" t="inlineStr">
         <is>
           <t>LEARN_MORE</t>
         </is>
       </c>
-      <c r="DJ4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>META_Leads_Recompo_Agenda_2026Q2</t>
@@ -1681,8 +1404,6 @@
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Outcome Leads</t>
@@ -1693,19 +1414,11 @@
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1716,35 +1429,21 @@
           <t>Prospeccion_Broad_GrupoA</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>&lt;TU_PAGE_ID&gt;</t>
-        </is>
-      </c>
       <c r="X5" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
           <t>ES, CL, UY, CR, PR, US</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
           <t>All</t>
@@ -1760,31 +1459,11 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr">
         <is>
           <t>Spanish</t>
         </is>
       </c>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
-      <c r="AX5" t="inlineStr"/>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
-      <c r="BB5" t="inlineStr"/>
-      <c r="BC5" t="inlineStr"/>
       <c r="BD5" t="inlineStr">
         <is>
           <t>OFFSITE_CONVERSIONS</t>
@@ -1795,42 +1474,11 @@
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="inlineStr"/>
-      <c r="BJ5" t="inlineStr"/>
-      <c r="BK5" t="inlineStr"/>
-      <c r="BL5" t="inlineStr"/>
-      <c r="BM5" t="inlineStr"/>
-      <c r="BN5" t="inlineStr"/>
-      <c r="BO5" t="inlineStr"/>
-      <c r="BP5" t="inlineStr"/>
-      <c r="BQ5" t="inlineStr"/>
-      <c r="BR5" t="inlineStr"/>
-      <c r="BS5" t="inlineStr"/>
-      <c r="BT5" t="inlineStr"/>
-      <c r="BU5" t="inlineStr"/>
-      <c r="BV5" t="inlineStr"/>
-      <c r="BW5" t="inlineStr"/>
-      <c r="BX5" t="inlineStr"/>
-      <c r="BY5" t="inlineStr"/>
-      <c r="BZ5" t="inlineStr"/>
-      <c r="CA5" t="inlineStr"/>
-      <c r="CB5" t="inlineStr"/>
-      <c r="CC5" t="inlineStr"/>
-      <c r="CD5" t="inlineStr"/>
-      <c r="CE5" t="inlineStr"/>
-      <c r="CF5" t="inlineStr"/>
-      <c r="CG5" t="inlineStr"/>
-      <c r="CH5" t="inlineStr"/>
-      <c r="CI5" t="inlineStr"/>
-      <c r="CJ5" t="inlineStr"/>
-      <c r="CK5" t="inlineStr"/>
       <c r="CL5" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1864,7 +1512,6 @@
           <t>salchichapro.com</t>
         </is>
       </c>
-      <c r="CR5" t="inlineStr"/>
       <c r="CS5" t="inlineStr">
         <is>
           <t>Video Page Post Ad</t>
@@ -1875,29 +1522,13 @@
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=recompo_agenda&amp;utm_content={{ad.name}}&amp;utm_term={{adset.name}}</t>
         </is>
       </c>
-      <c r="CU5" t="inlineStr"/>
-      <c r="CV5" t="inlineStr"/>
-      <c r="CW5" t="inlineStr"/>
-      <c r="CX5" t="inlineStr"/>
-      <c r="CY5" t="inlineStr"/>
-      <c r="CZ5" t="inlineStr"/>
-      <c r="DA5" t="inlineStr"/>
-      <c r="DB5" t="inlineStr"/>
-      <c r="DC5" t="inlineStr"/>
-      <c r="DD5" t="inlineStr"/>
-      <c r="DE5" t="inlineStr"/>
-      <c r="DF5" t="inlineStr"/>
-      <c r="DG5" t="inlineStr"/>
-      <c r="DH5" t="inlineStr"/>
       <c r="DI5" t="inlineStr">
         <is>
           <t>LEARN_MORE</t>
         </is>
       </c>
-      <c r="DJ5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>META_Leads_Recompo_Agenda_2026Q2</t>
@@ -1908,8 +1539,6 @@
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Outcome Leads</t>
@@ -1920,19 +1549,11 @@
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -1943,35 +1564,21 @@
           <t>Prospeccion_Broad_GrupoA</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>&lt;TU_PAGE_ID&gt;</t>
-        </is>
-      </c>
       <c r="X6" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
           <t>ES, CL, UY, CR, PR, US</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
           <t>All</t>
@@ -1987,31 +1594,11 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr">
         <is>
           <t>Spanish</t>
         </is>
       </c>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr"/>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
       <c r="BD6" t="inlineStr">
         <is>
           <t>OFFSITE_CONVERSIONS</t>
@@ -2022,42 +1609,11 @@
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="inlineStr"/>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="inlineStr"/>
-      <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
-      <c r="BQ6" t="inlineStr"/>
-      <c r="BR6" t="inlineStr"/>
-      <c r="BS6" t="inlineStr"/>
-      <c r="BT6" t="inlineStr"/>
-      <c r="BU6" t="inlineStr"/>
-      <c r="BV6" t="inlineStr"/>
-      <c r="BW6" t="inlineStr"/>
-      <c r="BX6" t="inlineStr"/>
-      <c r="BY6" t="inlineStr"/>
-      <c r="BZ6" t="inlineStr"/>
-      <c r="CA6" t="inlineStr"/>
-      <c r="CB6" t="inlineStr"/>
-      <c r="CC6" t="inlineStr"/>
-      <c r="CD6" t="inlineStr"/>
-      <c r="CE6" t="inlineStr"/>
-      <c r="CF6" t="inlineStr"/>
-      <c r="CG6" t="inlineStr"/>
-      <c r="CH6" t="inlineStr"/>
-      <c r="CI6" t="inlineStr"/>
-      <c r="CJ6" t="inlineStr"/>
-      <c r="CK6" t="inlineStr"/>
       <c r="CL6" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -2091,7 +1647,6 @@
           <t>salchichapro.com</t>
         </is>
       </c>
-      <c r="CR6" t="inlineStr"/>
       <c r="CS6" t="inlineStr">
         <is>
           <t>Video Page Post Ad</t>
@@ -2102,29 +1657,13 @@
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=recompo_agenda&amp;utm_content={{ad.name}}&amp;utm_term={{adset.name}}</t>
         </is>
       </c>
-      <c r="CU6" t="inlineStr"/>
-      <c r="CV6" t="inlineStr"/>
-      <c r="CW6" t="inlineStr"/>
-      <c r="CX6" t="inlineStr"/>
-      <c r="CY6" t="inlineStr"/>
-      <c r="CZ6" t="inlineStr"/>
-      <c r="DA6" t="inlineStr"/>
-      <c r="DB6" t="inlineStr"/>
-      <c r="DC6" t="inlineStr"/>
-      <c r="DD6" t="inlineStr"/>
-      <c r="DE6" t="inlineStr"/>
-      <c r="DF6" t="inlineStr"/>
-      <c r="DG6" t="inlineStr"/>
-      <c r="DH6" t="inlineStr"/>
       <c r="DI6" t="inlineStr">
         <is>
           <t>LEARN_MORE</t>
         </is>
       </c>
-      <c r="DJ6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>META_Leads_Recompo_Agenda_2026Q2</t>
@@ -2135,8 +1674,6 @@
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Outcome Leads</t>
@@ -2147,19 +1684,11 @@
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -2170,35 +1699,21 @@
           <t>Prospeccion_Broad_GrupoA</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>&lt;TU_PAGE_ID&gt;</t>
-        </is>
-      </c>
       <c r="X7" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr">
         <is>
           <t>ES, CL, UY, CR, PR, US</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
           <t>All</t>
@@ -2214,31 +1729,11 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr">
         <is>
           <t>Spanish</t>
         </is>
       </c>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
-      <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
       <c r="BD7" t="inlineStr">
         <is>
           <t>OFFSITE_CONVERSIONS</t>
@@ -2249,42 +1744,11 @@
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="BH7" t="inlineStr"/>
-      <c r="BI7" t="inlineStr"/>
-      <c r="BJ7" t="inlineStr"/>
-      <c r="BK7" t="inlineStr"/>
-      <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="inlineStr"/>
-      <c r="BN7" t="inlineStr"/>
-      <c r="BO7" t="inlineStr"/>
-      <c r="BP7" t="inlineStr"/>
-      <c r="BQ7" t="inlineStr"/>
-      <c r="BR7" t="inlineStr"/>
-      <c r="BS7" t="inlineStr"/>
-      <c r="BT7" t="inlineStr"/>
-      <c r="BU7" t="inlineStr"/>
-      <c r="BV7" t="inlineStr"/>
-      <c r="BW7" t="inlineStr"/>
-      <c r="BX7" t="inlineStr"/>
-      <c r="BY7" t="inlineStr"/>
-      <c r="BZ7" t="inlineStr"/>
-      <c r="CA7" t="inlineStr"/>
-      <c r="CB7" t="inlineStr"/>
-      <c r="CC7" t="inlineStr"/>
-      <c r="CD7" t="inlineStr"/>
-      <c r="CE7" t="inlineStr"/>
-      <c r="CF7" t="inlineStr"/>
-      <c r="CG7" t="inlineStr"/>
-      <c r="CH7" t="inlineStr"/>
-      <c r="CI7" t="inlineStr"/>
-      <c r="CJ7" t="inlineStr"/>
-      <c r="CK7" t="inlineStr"/>
       <c r="CL7" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -2318,7 +1782,6 @@
           <t>salchichapro.com</t>
         </is>
       </c>
-      <c r="CR7" t="inlineStr"/>
       <c r="CS7" t="inlineStr">
         <is>
           <t>Video Page Post Ad</t>
@@ -2329,33 +1792,13 @@
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=recompo_agenda&amp;utm_content={{ad.name}}&amp;utm_term={{adset.name}}</t>
         </is>
       </c>
-      <c r="CU7" t="inlineStr"/>
-      <c r="CV7" t="inlineStr"/>
-      <c r="CW7" t="inlineStr"/>
-      <c r="CX7" t="inlineStr"/>
-      <c r="CY7" t="inlineStr"/>
-      <c r="CZ7" t="inlineStr"/>
-      <c r="DA7" t="inlineStr"/>
-      <c r="DB7" t="inlineStr"/>
-      <c r="DC7" t="inlineStr"/>
-      <c r="DD7" t="inlineStr"/>
-      <c r="DE7" t="inlineStr"/>
-      <c r="DF7" t="inlineStr"/>
-      <c r="DG7" t="inlineStr"/>
-      <c r="DH7" t="inlineStr"/>
       <c r="DI7" t="inlineStr">
         <is>
           <t>LEARN_MORE</t>
-        </is>
-      </c>
-      <c r="DJ7" t="inlineStr">
-        <is>
-          <t>&lt;STORY_ID_MARCELO_1&gt;</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>META_Leads_Recompo_Agenda_2026Q2</t>
@@ -2366,8 +1809,6 @@
           <t>PAUSED</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Outcome Leads</t>
@@ -2378,19 +1819,11 @@
           <t>AUCTION</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -2401,35 +1834,21 @@
           <t>Prospeccion_Broad_GrupoA</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>&lt;TU_PAGE_ID&gt;</t>
-        </is>
-      </c>
       <c r="X8" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
           <t>ES, CL, UY, CR, PR, US</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
           <t>All</t>
@@ -2445,31 +1864,11 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr">
         <is>
           <t>Spanish</t>
         </is>
       </c>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
       <c r="BD8" t="inlineStr">
         <is>
           <t>OFFSITE_CONVERSIONS</t>
@@ -2480,42 +1879,11 @@
           <t>IMPRESSIONS</t>
         </is>
       </c>
-      <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="inlineStr">
         <is>
           <t>Highest volume or value</t>
         </is>
       </c>
-      <c r="BH8" t="inlineStr"/>
-      <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="inlineStr"/>
-      <c r="BK8" t="inlineStr"/>
-      <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="inlineStr"/>
-      <c r="BN8" t="inlineStr"/>
-      <c r="BO8" t="inlineStr"/>
-      <c r="BP8" t="inlineStr"/>
-      <c r="BQ8" t="inlineStr"/>
-      <c r="BR8" t="inlineStr"/>
-      <c r="BS8" t="inlineStr"/>
-      <c r="BT8" t="inlineStr"/>
-      <c r="BU8" t="inlineStr"/>
-      <c r="BV8" t="inlineStr"/>
-      <c r="BW8" t="inlineStr"/>
-      <c r="BX8" t="inlineStr"/>
-      <c r="BY8" t="inlineStr"/>
-      <c r="BZ8" t="inlineStr"/>
-      <c r="CA8" t="inlineStr"/>
-      <c r="CB8" t="inlineStr"/>
-      <c r="CC8" t="inlineStr"/>
-      <c r="CD8" t="inlineStr"/>
-      <c r="CE8" t="inlineStr"/>
-      <c r="CF8" t="inlineStr"/>
-      <c r="CG8" t="inlineStr"/>
-      <c r="CH8" t="inlineStr"/>
-      <c r="CI8" t="inlineStr"/>
-      <c r="CJ8" t="inlineStr"/>
-      <c r="CK8" t="inlineStr"/>
       <c r="CL8" t="inlineStr">
         <is>
           <t>PAUSED</t>
@@ -2549,7 +1917,6 @@
           <t>salchichapro.com</t>
         </is>
       </c>
-      <c r="CR8" t="inlineStr"/>
       <c r="CS8" t="inlineStr">
         <is>
           <t>Video Page Post Ad</t>
@@ -2560,28 +1927,9 @@
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=recompo_agenda&amp;utm_content={{ad.name}}&amp;utm_term={{adset.name}}</t>
         </is>
       </c>
-      <c r="CU8" t="inlineStr"/>
-      <c r="CV8" t="inlineStr"/>
-      <c r="CW8" t="inlineStr"/>
-      <c r="CX8" t="inlineStr"/>
-      <c r="CY8" t="inlineStr"/>
-      <c r="CZ8" t="inlineStr"/>
-      <c r="DA8" t="inlineStr"/>
-      <c r="DB8" t="inlineStr"/>
-      <c r="DC8" t="inlineStr"/>
-      <c r="DD8" t="inlineStr"/>
-      <c r="DE8" t="inlineStr"/>
-      <c r="DF8" t="inlineStr"/>
-      <c r="DG8" t="inlineStr"/>
-      <c r="DH8" t="inlineStr"/>
       <c r="DI8" t="inlineStr">
         <is>
           <t>LEARN_MORE</t>
-        </is>
-      </c>
-      <c r="DJ8" t="inlineStr">
-        <is>
-          <t>&lt;STORY_ID_MARCELO_2&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set real Page ID in Link Object ID for bulk import
https://claude.ai/code/session_01PamzbAcKurpbQ29kpfFhzA
</commit_message>
<xml_diff>
--- a/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
+++ b/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
@@ -1029,6 +1029,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>890534534153879</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
@@ -1164,6 +1169,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>890534534153879</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
@@ -1299,6 +1309,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>890534534153879</t>
+        </is>
+      </c>
       <c r="X4" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
@@ -1434,6 +1449,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>890534534153879</t>
+        </is>
+      </c>
       <c r="X5" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
@@ -1569,6 +1589,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>890534534153879</t>
+        </is>
+      </c>
       <c r="X6" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
@@ -1704,6 +1729,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>890534534153879</t>
+        </is>
+      </c>
       <c r="X7" t="inlineStr">
         <is>
           <t>https://salchichapro.com/metodorecomposicion</t>
@@ -1837,6 +1867,11 @@
       <c r="U8" t="inlineStr">
         <is>
           <t>50</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>890534534153879</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">

</xml_diff>

<commit_message>
Swap Marcelo ads to angle 4 (interconnected body) and angle 1 (dermatitis)
https://claude.ai/code/session_01PamzbAcKurpbQ29kpfFhzA
</commit_message>
<xml_diff>
--- a/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
+++ b/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
@@ -1786,25 +1786,24 @@
       </c>
       <c r="CM7" t="inlineStr">
         <is>
-          <t>Marcelo_Autoridad</t>
+          <t>Marcelo_CuerpoInterconectado</t>
         </is>
       </c>
       <c r="CN7" t="inlineStr">
         <is>
-          <t>Yo empiezo donde la medicina termina</t>
+          <t>Un solo cuerpo inflamado, no problemas separados</t>
         </is>
       </c>
       <c r="CO7" t="inlineStr">
         <is>
-          <t>Soy el Dr. Marcelo Hernán. Más de 20 años como veterinario y 6 sin darle un solo pellet a mis perros.
-En la universidad casi no se enseña nutrición de carnívoros, por eso tantos salchichas viven con problemas de piel, peso y digestión que no ceden con nada.
-Yo empiezo donde la medicina termina: resolviendo la causa desde el plato, con un plan individual y acompañamiento.
-Agenda tu llamada de evaluación, sin costo.</t>
+          <t>La picazón de tu Dachshund, sus gases, su ansiedad cuando te vas y su sobrepeso no son problemas distintos: es un solo cuerpo inflamado mandando señales en tres idiomas, intestino, piel y comportamiento.
+Soy el Dr. Marcelo Hernan. Con el Metodo Recomposicion Dachshund trabajo los 90 dias que hacen falta para apagar el incendio real, no el sintoma.
+Conoce el metodo definitivo para la salud de tu salchicha, desde la raiz.</t>
         </is>
       </c>
       <c r="CP7" t="inlineStr">
         <is>
-          <t>Nutrición natural individual para perros salchicha</t>
+          <t>Metodo de 90 dias, desde la raiz</t>
         </is>
       </c>
       <c r="CQ7" t="inlineStr">
@@ -1931,20 +1930,20 @@
       </c>
       <c r="CN8" t="inlineStr">
         <is>
-          <t>La dermatitis se resuelve desde la raíz</t>
+          <t>Apagan el sintoma, el incendio sigue adentro</t>
         </is>
       </c>
       <c r="CO8" t="inlineStr">
         <is>
-          <t>La piel roja, el rascado y la caída de pelo no son la temporada ni las pulgas. Son el grito de auxilio de tu salchicha.
-Tratar la piel sin cambiar el plato es como secar el piso con la llave abierta. Soy el Dr. Marcelo Hernán y te explico las 3 verdades sobre la dermatitis que casi nadie te cuenta.
-Resolvemos la causa, de adentro hacia afuera.
-Agenda tu llamada de evaluación, sin costo.</t>
+          <t>Croqueta premium, cremas dermatologicas, champu medicado, corticoides... y tu Dachshund sigue rascandose, sigue inflamado, sigue igual.
+No es porque seas mal dueno. Es porque ninguno de esos tratamientos toco la causa real: apagan el sintoma, pero el incendio sigue adentro.
+Soy el Dr. Marcelo Hernan, veterinario dedicado 100% al Dachshund. Diseno protocolos de recomposicion biologica para cada perro, sin farmacos y sin ensayo y error.
+Conoce el metodo definitivo para recuperar la salud de tu salchicha desde adentro.</t>
         </is>
       </c>
       <c r="CP8" t="inlineStr">
         <is>
-          <t>Un veterinario enfocado solo en perros salchicha</t>
+          <t>Veterinario enfocado solo en perros salchicha</t>
         </is>
       </c>
       <c r="CQ8" t="inlineStr">

</xml_diff>

<commit_message>
Set Marcelo ads to Dermatitis and IVDD angles
https://claude.ai/code/session_01PamzbAcKurpbQ29kpfFhzA
</commit_message>
<xml_diff>
--- a/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
+++ b/clientes/dachshund-salud/docs/Importacion-Masiva-Meta-Recomposicion.xlsx
@@ -1786,24 +1786,25 @@
       </c>
       <c r="CM7" t="inlineStr">
         <is>
-          <t>Marcelo_CuerpoInterconectado</t>
+          <t>Marcelo_Dermatitis</t>
         </is>
       </c>
       <c r="CN7" t="inlineStr">
         <is>
-          <t>Un solo cuerpo inflamado, no problemas separados</t>
+          <t>Apagan el síntoma, el incendio sigue adentro</t>
         </is>
       </c>
       <c r="CO7" t="inlineStr">
         <is>
-          <t>La picazón de tu Dachshund, sus gases, su ansiedad cuando te vas y su sobrepeso no son problemas distintos: es un solo cuerpo inflamado mandando señales en tres idiomas, intestino, piel y comportamiento.
-Soy el Dr. Marcelo Hernan. Con el Metodo Recomposicion Dachshund trabajo los 90 dias que hacen falta para apagar el incendio real, no el sintoma.
-Conoce el metodo definitivo para la salud de tu salchicha, desde la raiz.</t>
+          <t>Croqueta premium, cremas dermatológicas, champú medicado, corticoides... y tu Dachshund sigue rascándose, sigue inflamado, sigue igual.
+No es porque seas mal dueño. Es porque ninguno de esos tratamientos tocó la causa real: apagan el síntoma, pero el incendio sigue adentro.
+Soy el Dr. Marcelo Hernán, veterinario dedicado 100% al Dachshund. Diseño protocolos de recomposición biológica para cada perro, sin fármacos y sin ensayo y error.
+Conoce el método definitivo para recuperar la salud de tu salchicha desde adentro.</t>
         </is>
       </c>
       <c r="CP7" t="inlineStr">
         <is>
-          <t>Metodo de 90 dias, desde la raiz</t>
+          <t>Veterinario dedicado 100% al Dachshund</t>
         </is>
       </c>
       <c r="CQ7" t="inlineStr">
@@ -1925,25 +1926,26 @@
       </c>
       <c r="CM8" t="inlineStr">
         <is>
-          <t>Marcelo_Dermatitis</t>
+          <t>Marcelo_IVDD</t>
         </is>
       </c>
       <c r="CN8" t="inlineStr">
         <is>
-          <t>Apagan el sintoma, el incendio sigue adentro</t>
+          <t>La columna de tu salchicha empieza en el plato</t>
         </is>
       </c>
       <c r="CO8" t="inlineStr">
         <is>
-          <t>Croqueta premium, cremas dermatologicas, champu medicado, corticoides... y tu Dachshund sigue rascandose, sigue inflamado, sigue igual.
-No es porque seas mal dueno. Es porque ninguno de esos tratamientos toco la causa real: apagan el sintoma, pero el incendio sigue adentro.
-Soy el Dr. Marcelo Hernan, veterinario dedicado 100% al Dachshund. Diseno protocolos de recomposicion biologica para cada perro, sin farmacos y sin ensayo y error.
-Conoce el metodo definitivo para recuperar la salud de tu salchicha desde adentro.</t>
+          <t>Un día tu Dachshund salta del sofá como siempre. Al otro, no puede levantarse.
+No es un accidente: es el final de un proceso que empezó años antes, en el plato. 1 de cada 4 Dachshunds desarrolla IVDD, y casi nunca es solo genética: es inflamación crónica acumulada.
+La cadena es directa: croqueta, inflamación, sobrepeso, presión sobre la columna, disco herniado.
+Soy el Dr. Marcelo Hernán. Tengo un método de recomposición metabólica para construir músculo, bajar la inflamación y proteger su columna desde la nutrición, no desde el suplemento de turno.
+Conoce el método definitivo para proteger su salud antes de que sea tarde.</t>
         </is>
       </c>
       <c r="CP8" t="inlineStr">
         <is>
-          <t>Veterinario enfocado solo en perros salchicha</t>
+          <t>Protege su columna desde la nutrición</t>
         </is>
       </c>
       <c r="CQ8" t="inlineStr">

</xml_diff>